<commit_message>
Ultimos cambios realizados en el proyecto de asistencia, incluyendo modificaciones en archivos existentes y la adición de nuevos archivos para mejorar el seguimiento y registro de la asistencia. Se han actualizado los archivos de Excel relacionados con las vacaciones y permisos, así como el informe de asistencia. Además, se ha creado un nuevo archivo por lotes para automatizar ciertos procesos y un archivo de texto para almacenar registros adicionales.
</commit_message>
<xml_diff>
--- a/BUK/Buk vacaciones/BUK_vacaciones.xlsx
+++ b/BUK/Buk vacaciones/BUK_vacaciones.xlsx
@@ -61,21 +61,21 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Fecha Generación: 26/05/2026 a las 05:31PM</t>
+          <t>Fecha Generación: 28/05/2026 a las 02:34PM</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Fecha Desde: 25/05/2026</t>
+          <t>Fecha Desde: 27/05/2026</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Fecha Hasta: 26/05/2026</t>
+          <t>Fecha Hasta: 28/05/2026</t>
         </is>
       </c>
     </row>
@@ -110,18 +110,18 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>17.124.675-k</t>
+          <t>10.191.886-6</t>
         </is>
       </c>
       <c r="B7" s="1">
-        <v>46167.0</v>
+        <v>46169.0</v>
       </c>
       <c r="C7" t="n">
         <v>1.0</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>preaprobada</t>
+          <t>solicitada</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -137,14 +137,14 @@
         </is>
       </c>
       <c r="B8" s="1">
-        <v>46167.0</v>
+        <v>46169.0</v>
       </c>
       <c r="C8" t="n">
         <v>1.0</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>preaprobada</t>
+          <t>solicitada</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -156,46 +156,23 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>10.581.430-5</t>
+          <t>22.163.892-1</t>
         </is>
       </c>
       <c r="B9" s="1">
-        <v>46167.0</v>
+        <v>46170.0</v>
       </c>
       <c r="C9" t="n">
         <v>1.0</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>aprobada</t>
+          <t>solicitada</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Progresivas</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>9.854.831-9</t>
-        </is>
-      </c>
-      <c r="B10" s="1">
-        <v>46168.0</v>
-      </c>
-      <c r="C10" t="n">
-        <v>1.0</v>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>solicitada</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Progresivas</t>
+          <t>Legales</t>
         </is>
       </c>
     </row>

</xml_diff>